<commit_message>
feitas alterações no BD e em modelos.
</commit_message>
<xml_diff>
--- a/db/Dicionário_dados.xlsx
+++ b/db/Dicionário_dados.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="20417"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\DESENVOLVIMENTO\WORKSYNC\RepairIQ\db\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aluno\Documents\Julio\RepairIQ\db\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93C907F4-4B90-496D-BBA7-1EEEB2738CDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C346F54-EB2A-43E0-A3E6-019DF09CA413}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5040" yWindow="2520" windowWidth="21600" windowHeight="11205" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5040" yWindow="2520" windowWidth="10320" windowHeight="5025" firstSheet="2" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Relacionamento" sheetId="4" r:id="rId1"/>
@@ -26,24 +26,11 @@
     <sheet name="Planilha1" sheetId="22" r:id="rId11"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="368" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="367" uniqueCount="152">
   <si>
     <t>Relacionamento</t>
   </si>
@@ -303,9 +290,6 @@
     <t>senha</t>
   </si>
   <si>
-    <t>64 bytes</t>
-  </si>
-  <si>
     <t>login</t>
   </si>
   <si>
@@ -499,6 +483,9 @@
   </si>
   <si>
     <t>Total de bytes da tabela:</t>
+  </si>
+  <si>
+    <t>ativo</t>
   </si>
 </sst>
 </file>
@@ -956,40 +943,40 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1028,9 +1015,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1068,9 +1055,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1103,9 +1090,26 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1138,9 +1142,26 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1331,18 +1352,18 @@
       </c>
     </row>
     <row r="3" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="43" t="s">
+      <c r="A3" s="35" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="44"/>
-      <c r="C3" s="44"/>
-      <c r="D3" s="44"/>
+      <c r="B3" s="36"/>
+      <c r="C3" s="36"/>
+      <c r="D3" s="36"/>
     </row>
     <row r="4" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="45"/>
-      <c r="B4" s="46"/>
-      <c r="C4" s="46"/>
-      <c r="D4" s="46"/>
+      <c r="A4" s="37"/>
+      <c r="B4" s="38"/>
+      <c r="C4" s="38"/>
+      <c r="D4" s="38"/>
     </row>
     <row r="5" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
@@ -1359,7 +1380,7 @@
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="40" t="s">
+      <c r="A6" s="39" t="s">
         <v>10</v>
       </c>
       <c r="B6" s="22" t="s">
@@ -1368,22 +1389,22 @@
       <c r="C6" s="22" t="s">
         <v>13</v>
       </c>
-      <c r="D6" s="35" t="s">
+      <c r="D6" s="42" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="42"/>
+      <c r="A7" s="40"/>
       <c r="B7" s="22" t="s">
         <v>12</v>
       </c>
       <c r="C7" s="22" t="s">
         <v>13</v>
       </c>
-      <c r="D7" s="37"/>
+      <c r="D7" s="43"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="40" t="s">
+      <c r="A8" s="39" t="s">
         <v>14</v>
       </c>
       <c r="B8" s="22" t="s">
@@ -1392,7 +1413,7 @@
       <c r="C8" s="23" t="s">
         <v>31</v>
       </c>
-      <c r="D8" s="35" t="s">
+      <c r="D8" s="42" t="s">
         <v>40</v>
       </c>
     </row>
@@ -1404,7 +1425,7 @@
       <c r="C9" s="23" t="s">
         <v>13</v>
       </c>
-      <c r="D9" s="36"/>
+      <c r="D9" s="44"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="41"/>
@@ -1414,7 +1435,7 @@
       <c r="C10" s="23" t="s">
         <v>18</v>
       </c>
-      <c r="D10" s="36"/>
+      <c r="D10" s="44"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="41"/>
@@ -1424,40 +1445,40 @@
       <c r="C11" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="D11" s="36"/>
+      <c r="D11" s="44"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="42"/>
+      <c r="A12" s="40"/>
       <c r="B12" s="22" t="s">
         <v>17</v>
       </c>
       <c r="C12" s="22" t="s">
         <v>13</v>
       </c>
-      <c r="D12" s="37"/>
+      <c r="D12" s="43"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="40" t="s">
+      <c r="A13" s="39" t="s">
         <v>16</v>
       </c>
-      <c r="B13" s="35" t="s">
+      <c r="B13" s="42" t="s">
         <v>11</v>
       </c>
-      <c r="C13" s="35" t="s">
+      <c r="C13" s="42" t="s">
         <v>19</v>
       </c>
-      <c r="D13" s="35" t="s">
+      <c r="D13" s="42" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="42"/>
-      <c r="B14" s="37"/>
-      <c r="C14" s="37"/>
-      <c r="D14" s="37"/>
+      <c r="A14" s="40"/>
+      <c r="B14" s="43"/>
+      <c r="C14" s="43"/>
+      <c r="D14" s="43"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="40" t="s">
+      <c r="A15" s="39" t="s">
         <v>15</v>
       </c>
       <c r="B15" s="24" t="s">
@@ -1466,7 +1487,7 @@
       <c r="C15" s="22" t="s">
         <v>18</v>
       </c>
-      <c r="D15" s="35" t="s">
+      <c r="D15" s="42" t="s">
         <v>34</v>
       </c>
     </row>
@@ -1478,7 +1499,7 @@
       <c r="C16" s="22" t="s">
         <v>23</v>
       </c>
-      <c r="D16" s="36"/>
+      <c r="D16" s="44"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="41"/>
@@ -1488,7 +1509,7 @@
       <c r="C17" s="22" t="s">
         <v>24</v>
       </c>
-      <c r="D17" s="36"/>
+      <c r="D17" s="44"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="41"/>
@@ -1498,40 +1519,40 @@
       <c r="C18" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="D18" s="36"/>
+      <c r="D18" s="44"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="42"/>
+      <c r="A19" s="40"/>
       <c r="B19" s="24" t="s">
         <v>22</v>
       </c>
       <c r="C19" s="22" t="s">
         <v>26</v>
       </c>
-      <c r="D19" s="37"/>
+      <c r="D19" s="43"/>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="40" t="s">
+      <c r="A20" s="39" t="s">
         <v>21</v>
       </c>
-      <c r="B20" s="35" t="s">
+      <c r="B20" s="42" t="s">
         <v>15</v>
       </c>
-      <c r="C20" s="35" t="s">
+      <c r="C20" s="42" t="s">
         <v>25</v>
       </c>
-      <c r="D20" s="35" t="s">
+      <c r="D20" s="42" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="42"/>
-      <c r="B21" s="37"/>
-      <c r="C21" s="37"/>
-      <c r="D21" s="37"/>
+      <c r="A21" s="40"/>
+      <c r="B21" s="43"/>
+      <c r="C21" s="43"/>
+      <c r="D21" s="43"/>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="38" t="s">
+      <c r="A22" s="45" t="s">
         <v>17</v>
       </c>
       <c r="B22" s="24" t="s">
@@ -1540,19 +1561,19 @@
       <c r="C22" s="22" t="s">
         <v>23</v>
       </c>
-      <c r="D22" s="35" t="s">
+      <c r="D22" s="42" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="38"/>
+      <c r="A23" s="45"/>
       <c r="B23" s="24" t="s">
         <v>11</v>
       </c>
       <c r="C23" s="22" t="s">
         <v>18</v>
       </c>
-      <c r="D23" s="37"/>
+      <c r="D23" s="43"/>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="25" t="s">
@@ -1569,47 +1590,47 @@
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="35" t="s">
+      <c r="A25" s="42" t="s">
         <v>12</v>
       </c>
       <c r="B25" s="24"/>
       <c r="C25" s="22"/>
-      <c r="D25" s="35" t="s">
+      <c r="D25" s="42" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" s="36"/>
+      <c r="A26" s="44"/>
       <c r="B26" s="24" t="s">
         <v>10</v>
       </c>
       <c r="C26" s="22" t="s">
         <v>28</v>
       </c>
-      <c r="D26" s="36"/>
+      <c r="D26" s="44"/>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" s="36"/>
+      <c r="A27" s="44"/>
       <c r="B27" s="22" t="s">
         <v>27</v>
       </c>
       <c r="C27" s="22" t="s">
         <v>29</v>
       </c>
-      <c r="D27" s="36"/>
+      <c r="D27" s="44"/>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" s="37"/>
+      <c r="A28" s="43"/>
       <c r="B28" s="22" t="s">
         <v>15</v>
       </c>
       <c r="C28" s="22" t="s">
         <v>26</v>
       </c>
-      <c r="D28" s="37"/>
+      <c r="D28" s="43"/>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29" s="38" t="s">
+      <c r="A29" s="45" t="s">
         <v>30</v>
       </c>
       <c r="B29" s="24" t="s">
@@ -1618,22 +1639,22 @@
       <c r="C29" s="22" t="s">
         <v>31</v>
       </c>
-      <c r="D29" s="39" t="s">
+      <c r="D29" s="46" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A30" s="38"/>
+      <c r="A30" s="45"/>
       <c r="B30" s="24"/>
       <c r="C30" s="22"/>
-      <c r="D30" s="39"/>
+      <c r="D30" s="46"/>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="25"/>
       <c r="B31" s="24"/>
       <c r="C31" s="22"/>
       <c r="D31" s="22" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
@@ -1650,13 +1671,6 @@
     </row>
   </sheetData>
   <mergeCells count="21">
-    <mergeCell ref="A3:D4"/>
-    <mergeCell ref="A6:A7"/>
-    <mergeCell ref="A13:A14"/>
-    <mergeCell ref="A8:A12"/>
-    <mergeCell ref="D13:D14"/>
-    <mergeCell ref="D6:D7"/>
-    <mergeCell ref="D8:D12"/>
     <mergeCell ref="D15:D19"/>
     <mergeCell ref="A29:A30"/>
     <mergeCell ref="D29:D30"/>
@@ -1671,6 +1685,13 @@
     <mergeCell ref="A22:A23"/>
     <mergeCell ref="D22:D23"/>
     <mergeCell ref="D25:D28"/>
+    <mergeCell ref="A3:D4"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="A13:A14"/>
+    <mergeCell ref="A8:A12"/>
+    <mergeCell ref="D13:D14"/>
+    <mergeCell ref="D6:D7"/>
+    <mergeCell ref="D8:D12"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -1731,30 +1752,30 @@
         <v>48</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D6" s="4" t="s">
         <v>57</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="18" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>49</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D7" s="12" t="s">
         <v>58</v>
       </c>
       <c r="E7" s="11" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
@@ -1787,7 +1808,7 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
   </sheetData>
@@ -1861,13 +1882,13 @@
         <v>48</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D6" s="4" t="s">
         <v>57</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -1972,19 +1993,19 @@
     </row>
     <row r="13" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="19" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B13" s="10" t="s">
         <v>48</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D13" s="12" t="s">
         <v>58</v>
       </c>
       <c r="E13" s="11" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
@@ -2061,13 +2082,13 @@
         <v>48</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D6" s="4" t="s">
         <v>57</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -2157,7 +2178,7 @@
     </row>
     <row r="12" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="19" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B12" s="10" t="s">
         <v>48</v>
@@ -2169,12 +2190,12 @@
         <v>73</v>
       </c>
       <c r="E12" s="11" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="13" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B13" s="14" t="s">
         <v>48</v>
@@ -2186,24 +2207,24 @@
         <v>73</v>
       </c>
       <c r="E13" s="17" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="13" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B14" s="14" t="s">
         <v>48</v>
       </c>
       <c r="C14" s="15" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D14" s="16" t="s">
         <v>73</v>
       </c>
       <c r="E14" s="17" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
@@ -2215,7 +2236,7 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
   </sheetData>
@@ -2280,13 +2301,13 @@
         <v>48</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D6" s="4" t="s">
         <v>57</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -2294,7 +2315,7 @@
         <v>68</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>70</v>
@@ -2421,13 +2442,13 @@
         <v>48</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D6" s="4" t="s">
         <v>57</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -2437,31 +2458,31 @@
       <c r="B7" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="C7" s="4" t="s">
-        <v>52</v>
+      <c r="C7" s="4">
+        <v>40</v>
       </c>
       <c r="D7" s="12" t="s">
         <v>58</v>
       </c>
       <c r="E7" s="11" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="18" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B8" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="C8" s="4" t="s">
-        <v>70</v>
+      <c r="C8" s="4">
+        <v>20</v>
       </c>
       <c r="D8" s="12" t="s">
         <v>58</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
@@ -2471,20 +2492,26 @@
       <c r="B9" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="C9" s="4" t="s">
-        <v>86</v>
+      <c r="C9" s="4">
+        <v>64</v>
       </c>
       <c r="D9" s="12" t="s">
         <v>58</v>
       </c>
       <c r="E9" s="11" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="19"/>
-      <c r="B10" s="10"/>
-      <c r="C10" s="4"/>
+      <c r="A10" s="19" t="s">
+        <v>151</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="C10" s="4">
+        <v>1</v>
+      </c>
       <c r="D10" s="12"/>
       <c r="E10" s="11"/>
     </row>
@@ -2497,7 +2524,7 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
   </sheetData>
@@ -2568,12 +2595,12 @@
         <v>57</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="18" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>49</v>
@@ -2585,12 +2612,12 @@
         <v>58</v>
       </c>
       <c r="E7" s="11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="18" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B8" s="10" t="s">
         <v>49</v>
@@ -2602,12 +2629,12 @@
         <v>58</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="18" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B9" s="10" t="s">
         <v>49</v>
@@ -2619,12 +2646,12 @@
         <v>58</v>
       </c>
       <c r="E9" s="11" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="19" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B10" s="10" t="s">
         <v>48</v>
@@ -2636,12 +2663,12 @@
         <v>58</v>
       </c>
       <c r="E10" s="11" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="30" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B11" s="31" t="s">
         <v>48</v>
@@ -2653,7 +2680,7 @@
         <v>58</v>
       </c>
       <c r="E11" s="34" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2665,7 +2692,7 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B15">
         <f>SUM(C6:C11)</f>
@@ -2734,18 +2761,18 @@
         <v>48</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D6" s="4" t="s">
         <v>57</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="18" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>69</v>
@@ -2757,29 +2784,29 @@
         <v>58</v>
       </c>
       <c r="E7" s="11" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="18" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B8" s="10" t="s">
         <v>49</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D8" s="12" t="s">
         <v>58</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="18" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B9" s="10" t="s">
         <v>49</v>
@@ -2791,7 +2818,7 @@
         <v>58</v>
       </c>
       <c r="E9" s="11" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
@@ -2808,12 +2835,12 @@
         <v>58</v>
       </c>
       <c r="E10" s="11" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="30" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B11" s="31" t="s">
         <v>48</v>
@@ -2825,12 +2852,12 @@
         <v>73</v>
       </c>
       <c r="E11" s="34" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="13" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B12" s="14" t="s">
         <v>48</v>
@@ -2842,12 +2869,12 @@
         <v>73</v>
       </c>
       <c r="E12" s="17" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
   </sheetData>
@@ -2912,18 +2939,18 @@
         <v>48</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D6" s="4" t="s">
         <v>57</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="18" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>49</v>
@@ -2935,12 +2962,12 @@
         <v>58</v>
       </c>
       <c r="E7" s="11" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="18" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B8" s="10" t="s">
         <v>69</v>
@@ -2952,12 +2979,12 @@
         <v>58</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="18" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B9" s="10" t="s">
         <v>49</v>
@@ -2969,12 +2996,12 @@
         <v>58</v>
       </c>
       <c r="E9" s="11" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="19" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B10" s="10" t="s">
         <v>48</v>
@@ -2986,7 +3013,7 @@
         <v>73</v>
       </c>
       <c r="E10" s="11" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2998,7 +3025,7 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
   </sheetData>
@@ -3063,52 +3090,52 @@
         <v>48</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D6" s="4" t="s">
         <v>57</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="18" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B7" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="C7" s="4" t="s">
         <v>124</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="D7" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="E7" s="11" t="s">
         <v>125</v>
-      </c>
-      <c r="D7" s="12" t="s">
-        <v>58</v>
-      </c>
-      <c r="E7" s="11" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="18" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B8" s="10" t="s">
         <v>50</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D8" s="12" t="s">
         <v>58</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="18" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B9" s="10" t="s">
         <v>48</v>
@@ -3120,7 +3147,7 @@
         <v>73</v>
       </c>
       <c r="E9" s="11" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
@@ -3139,7 +3166,7 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
   </sheetData>

</xml_diff>